<commit_message>
feat(F-NAR-019): ATOM-DIF.ENE.001-04 Le soleil du grand pinceau
Réécriture vocale example4 : éclat de chiffon, énergie vécue.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.ENE.001-04.xlsx
+++ b/stories/arbres/ATOM-DIF.ENE.001-04.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>atelier peinture à la maison</t>
+          <t>atelier peinture : chiffon bleu, papier, fenêtre, tube jaune, grand pinceau bleu, pots, évier</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nino veut peindre un soleil jaune avec le grand pinceau bleu. Victorino arrive avec beaucoup d'énergie. Une goutte tombe. Ils jouent, ils attendent, Nino demande à maman. Le soleil est sur la feuille.</t>
+          <t>Une virgule jaune colle au bouchon. Sur le chiffon bleu, un éclat de chiffon brille. Nino veut le grand pinceau, maintenant, pour un soleil. Victorino saute, lève trop vite : une tache, le papier part. Sourire parti. Nino refuse de foncer, file des pots. Victorino veut passer. Nino appelle maman. Évier froid. Merci vécu. L'éclat de chiffon tient.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le tube jaune a un bouchon collant. Papa le tourne. Une petite virgule de peinture sort. Elle sent le papier neuf. Un chiffon bleu sèche près de la fenêtre. Le papier craque tout doucement. Tu sens la peinture, Nino ? Oui. Ça sent le papier. Maman pose de grandes feuilles. On a de la place, tous les deux. En ce moment, Nino regarde la feuille vide. Elle est un peu rugueuse. Je veux le grand pinceau. Pour un soleil. Il est dans le pot bleu. Le pot fait un petit clac. L'eau du pot est trouble. Victorino arrive en sautant. Il a beaucoup d'énergie. Il tourne. Il s'arrête. Il recommence. Il saute, papa. C'est son énergie. Ce n'est pas une faute. Victorino prend le grand pinceau bleu. Il veut peindre tout de suite. Une goutte jaune tombe sur la table. Elle fait un petit point brillant. À tour de rôle. Oui. On attend son tour. Le pinceau tremble un peu. Victorino ne le pose pas encore. Nino regarde maman.</t>
+          <t>Une virgule jaune colle au bouchon. Papa tourne le tube jaune. Elle colle, papa ! Tu la sens, sur tes doigts ? Oui, elle est froide. Ça sent le papier neuf, un peu. Tu le sens, Nino ? Oui, papa. Ça sent le papier. Un chiffon bleu sèche près de la fenêtre. Il pend, maman. Tu le vois, le chiffon ? Oui, il est mouillé. Sur le bleu, un éclat de chiffon brille. Il brille, papa ! Tu le vois, ce petit point ? Oui, un petit point. Maman pose de grandes feuilles. Elles sont rudes, maman. On a de la place, tous les deux. Oui, maman. Le coin des pots est libre, Nino ? Oui, papa. Le pot bleu fait un petit clac. L'eau est trouble. L'eau du pot, Nino ? Oui, elle bouge. Le grand pinceau est dans le pot ? Oui, il est bleu. En ce moment, Nino veut le grand pinceau. Je veux le grand pinceau, maintenant ! Pour un soleil, maman. Un grand soleil jaune ? Oui, toute la feuille. Avec Victorino, Nino ? Oui, papa. Victorino arrive en sautant. Victorino ! J'arrive ! Il tourne près de la table. Ses pieds tapent le sol, fort. Il saute, papa. Tu le vois sauter, toi ? Oui, beaucoup. Ses mains bougent vite, Nino ? Oui, maman. Le pinceau ! Victorino prend le grand pinceau bleu. Il le lève trop vite. Oh ! Une goutte jaune tombe sur la table. Ça tache ! Le papier glisse vers le bord. Il part ! Vite ! Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu, lourdes. Maman s'accroupit à la même hauteur. Tu veux le soleil avec Victorino ? Oui, maman. Tes mains sont collantes, Nino ? Un peu, papa. Nino refuse de foncer. Il referme les mains. Personne ne parle. Il observe le chiffon, un instant. L'éclat de chiffon tremble, puis tient. L'éclat, papa ? Tu le vois, toi ? Oui, sur le bleu. Moi, le pinceau. Le pinceau tremble dans sa main. Victorino ne le pose pas. Nino regarde maman.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le tube jaune a un bouchon collant. Papa le tourne. Une petite virgule de peinture sort. Elle sent le papier neuf. Un chiffon bleu sèche près de la fenêtre. Le papier craque tout doucement. Tu sens la peinture, Nino ? Oui. Ça sent le papier. Maman pose de grandes feuilles. On a de la place, tous les deux. En ce moment, Nino regarde la feuille vide. Elle est un peu rugueuse. Je veux le grand pinceau. Pour un soleil. Il est dans le pot bleu. Le pot fait un petit clac. L'eau du pot est trouble. Victorino arrive en sautant. Il a beaucoup d'énergie. Il tourne. Il s'arrête. Il recommence. Il saute, papa. C'est son énergie. Ce n'est pas une faute. Victorino prend le grand pinceau bleu. Il veut peindre tout de suite. Une goutte jaune tombe sur la table. Elle fait un petit point brillant. À tour de rôle. Oui. On attend son tour. Le pinceau tremble un peu. Victorino ne le pose pas encore. Nino regarde maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une virgule jaune colle au bouchon. Papa tourne le tube jaune. Elle colle, papa ! Tu la sens, sur tes doigts ? Oui, elle est froide. Ça sent le papier neuf, un peu. Tu le sens, Nino ? Oui, papa. Ça sent le papier. Un chiffon bleu sèche près de la fenêtre. Il pend, maman. Tu le vois, le chiffon ? Oui, il est mouillé. Sur le bleu, un &lt;emphasis level="moderate"&gt;éclat de chiffon&lt;/emphasis&gt; brille. Il brille, papa ! Tu le vois, ce petit point ? Oui, un petit point. Maman pose de grandes feuilles. Elles sont rudes, maman. On a de la place, tous les deux. Oui, maman. Le coin des pots est libre, Nino ? Oui, papa. Le pot bleu fait un petit clac. L'eau est trouble. L'eau du pot, Nino ? Oui, elle bouge. Le grand pinceau est dans le pot ? Oui, il est bleu. En ce moment, Nino veut le grand pinceau. Je veux le grand pinceau, maintenant ! Pour un soleil, maman. Un grand soleil jaune ? Oui, toute la feuille. Avec Victorino, Nino ? Oui, papa. Victorino arrive en sautant. Victorino ! J'arrive ! Il tourne près de la table. Ses pieds tapent le sol, fort. Il saute, papa. Tu le vois sauter, toi ? Oui, beaucoup. Ses mains bougent vite, Nino ? Oui, maman. Le pinceau ! Victorino prend le grand pinceau bleu. Il le lève trop vite. Oh ! Une goutte jaune tombe sur la table. Ça tache ! Le papier glisse vers le bord. Il part ! Vite ! Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu, lourdes. Maman s'accroupit à la même hauteur. Tu veux le soleil avec Victorino ? Oui, maman. Tes mains sont collantes, Nino ? Un peu, papa. Nino refuse de foncer. Il referme les mains. Personne ne parle. Il observe le chiffon, un instant. L'éclat de chiffon tremble, puis tient. L'éclat, papa ? Tu le vois, toi ? Oui, sur le bleu. Moi, le pinceau. Le pinceau tremble dans sa main. Victorino ne le pose pas. Nino regarde maman.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Mila est à l'atelier peinture. Maman a posé des feuilles. Rayan arrive en sautant. Il a beaucoup d'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Il tourne, il s'arrête, il recommence. Le pinceau tremble dans sa main. Mila le regarde. Maman est près de la table. Elle dit : beaucoup d'énergie, ce n'est pas une faute. On peut jouer. On peut attendre. On peut demander à un adulte. Mila hoche la tête. Il y a un grand pinceau bleu. Rayan le prend. Il veut peindre tout de suite. Mila dit : à tour de rôle. Rayan pose le pinceau. Il attend son tour. Puis Mila peint un rond. Rayan saute sur place, un peu. L'énergie est encore là. Ce n'est pas une faute. Mila dit : maintenant c'est toi. Rayan joue. Il peint une ligne. Après, ils font une file pour les pots. Rayan a envie d'aller vite. Mila dit : on peut attendre. Rayan souffle. Il reste dans la file. Parce qu'ils attendent, chacun a de la peinture. Ils jouent. Plus tard, Rayan a encore trop d'énergie pour la chaise. Mila va vers maman. Elle demande à un adulte. Maman dit : Rayan, viens marcher avec moi jusqu'à l'évier. Rayan marche. Il pose les mains sous l'eau. L'eau est froide. Il se calme un peu. Mila l'attend. Puis ils rincent les pinceaux ensemble. Maman dit : ce n'est pas une faute. Vous avez pu jouer ou attendre. [pause]</t>
+          <t>Une virgule jaune colle au bouchon. Papa tourne le tube jaune. Elle colle, papa ! Tu la sens, sur tes doigts ? Oui, elle est froide. Ça sent le papier neuf, un peu. Tu le sens, Nino ? Oui, papa. Ça sent le papier. Un chiffon bleu sèche près de la fenêtre. Il pend, maman. Tu le vois, le chiffon ? Oui, il est mouillé. Sur le bleu, un &lt;emphasis&gt;éclat de chiffon&lt;/emphasis&gt; brille. Il brille, papa ! Tu le vois, ce petit point ? Oui, un petit point. Maman pose de grandes feuilles. Elles sont rudes, maman. On a de la place, tous les deux. Oui, maman. Le coin des pots est libre, Nino ? Oui, papa. Le pot bleu fait un petit clac. L'eau est trouble. L'eau du pot, Nino ? Oui, elle bouge. Le grand pinceau est dans le pot ? Oui, il est bleu. En ce moment, Nino veut le grand pinceau. Je veux le grand pinceau, maintenant ! Pour un soleil, maman. Un grand soleil jaune ? Oui, toute la feuille. Avec Victorino, Nino ? Oui, papa. Victorino arrive en sautant. Victorino ! J'arrive ! Il tourne près de la table. Ses pieds tapent le sol, fort. Il saute, papa. Tu le vois sauter, toi ? Oui, beaucoup. Ses mains bougent vite, Nino ? Oui, maman. Le pinceau ! Victorino prend le grand pinceau bleu. Il le lève trop vite. Oh ! Une goutte jaune tombe sur la table. Ça tache ! Le papier glisse vers le bord. Il part ! Vite ! Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu, lourdes. Maman s'accroupit à la même hauteur. Tu veux le soleil avec Victorino ? Oui, maman. Tes mains sont collantes, Nino ? Un peu, papa. Nino refuse de foncer. Il referme les mains. Personne ne parle. Il observe le chiffon, un instant. L'éclat de chiffon tremble, puis tient. L'éclat, papa ? Tu le vois, toi ? Oui, sur le bleu. Moi, le pinceau. Le pinceau tremble dans sa main. Victorino ne le pose pas. Nino regarde maman. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>énergie</t>
+          <t>éclat de chiffon</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,45 +1321,93 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_grand_pinceau_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le tube jaune a un bouchon collant.
-narrateur|Papa le tourne.
-narrateur|Une petite virgule de peinture sort.
-narrateur|Elle sent le papier neuf.
+          <t>narrateur|Une virgule jaune colle au bouchon.
+narrateur|Papa tourne le tube jaune.
+enfant-m|Elle colle, papa !
+papa|Tu la sens, sur tes doigts ?
+enfant-m|Oui, elle est froide.
+narrateur|Ça sent le papier neuf, un peu.
+papa|Tu le sens, Nino ?
+enfant-m|Oui, papa.
+enfant-m|Ça sent le papier.
 narrateur|Un chiffon bleu sèche près de la fenêtre.
-narrateur|Le papier craque tout doucement.
-papa|Tu sens la peinture, Nino ?
-enfant-m|Oui.
-enfant-m|Ça sent le papier.
+enfant-m|Il pend, maman.
+maman|Tu le vois, le chiffon ?
+enfant-m|Oui, il est mouillé.
+narrateur|Sur le bleu, un éclat de chiffon brille.
+enfant-m|Il brille, papa !
+papa|Tu le vois, ce petit point ?
+enfant-m|Oui, un petit point.
 narrateur|Maman pose de grandes feuilles.
+enfant-m|Elles sont rudes, maman.
 maman|On a de la place, tous les deux.
-narrateur|En ce moment, Nino regarde la feuille vide.
-narrateur|Elle est un peu rugueuse.
-enfant-m|Je veux le grand pinceau.
-enfant-m|Pour un soleil.
-maman|Il est dans le pot bleu.
-narrateur|Le pot fait un petit clac.
-narrateur|L'eau du pot est trouble.
+enfant-m|Oui, maman.
+papa|Le coin des pots est libre, Nino ?
+enfant-m|Oui, papa.
+narrateur|Le pot bleu fait un petit clac.
+enfant-m|L'eau est trouble.
+papa|L'eau du pot, Nino ?
+enfant-m|Oui, elle bouge.
+maman|Le grand pinceau est dans le pot ?
+enfant-m|Oui, il est bleu.
+narrateur|En ce moment, Nino veut le grand pinceau.
+enfant-m|Je veux le grand pinceau, maintenant !
+enfant-m|Pour un soleil, maman.
+maman|Un grand soleil jaune ?
+enfant-m|Oui, toute la feuille.
+papa|Avec Victorino, Nino ?
+enfant-m|Oui, papa.
 narrateur|Victorino arrive en sautant.
-narrateur|Il a beaucoup d'énergie.
-narrateur|Il tourne.
-narrateur|Il s'arrête.
-narrateur|Il recommence.
+enfant-m|Victorino !
+copain|J'arrive !
+narrateur|Il tourne près de la table.
+narrateur|Ses pieds tapent le sol, fort.
 enfant-m|Il saute, papa.
-papa|C'est son énergie.
-papa|Ce n'est pas une faute.
+papa|Tu le vois sauter, toi ?
+enfant-m|Oui, beaucoup.
+maman|Ses mains bougent vite, Nino ?
+enfant-m|Oui, maman.
+copain|Le pinceau !
 narrateur|Victorino prend le grand pinceau bleu.
-narrateur|Il veut peindre tout de suite.
+narrateur|Il le lève trop vite.
+enfant-m|Oh !
 narrateur|Une goutte jaune tombe sur la table.
-narrateur|Elle fait un petit point brillant.
-enfant-m|À tour de rôle.
-maman|Oui.
-maman|On attend son tour.
-narrateur|Le pinceau tremble un peu.
-narrateur|Victorino ne le pose pas encore.
+enfant-m|Ça tache !
+narrateur|Le papier glisse vers le bord.
+enfant-m|Il part !
+copain|Vite !
+narrateur|Le sourire de Nino disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu, lourdes.
+narrateur|Maman s'accroupit à la même hauteur.
+maman|Tu veux le soleil avec Victorino ?
+enfant-m|Oui, maman.
+papa|Tes mains sont collantes, Nino ?
+enfant-m|Un peu, papa.
+narrateur|Nino refuse de foncer.
+narrateur|Il referme les mains.
+narrateur|Personne ne parle.
+narrateur|Il observe le chiffon, un instant.
+narrateur|L'éclat de chiffon tremble, puis tient.
+enfant-m|L'éclat, papa ?
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur le bleu.
+copain|Moi, le pinceau.
+narrateur|Le pinceau tremble dans sa main.
+narrateur|Victorino ne le pose pas.
 narrateur|Nino regarde maman.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>peinture,papier</t>
         </is>
       </c>
     </row>
@@ -1391,12 +1439,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorino a de l'énergie. Que peut-on faire ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorino a de l'&lt;emphasis level="moderate"&gt;énergie&lt;/emphasis&gt;. Que peut-on faire ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Rayan a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Que peut-on faire ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorino a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Que peut-on faire ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1406,7 +1454,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>jouer | attendre | un adulte | demander</t>
+          <t>jouer | attendre | un adulte | jouer ou attendre | demander</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1459,7 +1507,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1470,7 +1518,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1485,11 +1533,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1500,23 +1548,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1531,17 +1579,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=victorino_saute_que_peut_on_faire; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1574,17 +1622,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nino va vers maman. Maman, on fait quoi ? On peint, tous les deux. On attend le pinceau. Tu m'as appelée, Nino. Victorino, viens marcher jusqu'à l'évier. Victorino marche. Il pose les mains sous l'eau. L'eau est froide. Il souffle. Il se calme un peu. L'énergie est encore là. Ce n'est pas une faute. On attend. Victorino pose le pinceau dans le pot. Il attend son tour. C'est à Nino. Nino prend le grand pinceau bleu. Il peint un rond. Le rond est jaune comme un soleil. Maintenant c'est toi. Victorino peint une ligne. La ligne part du rond. C'est un rayon. Après, ils font une file pour les pots. Victorino a envie d'aller vite. On peut attendre. Victorino souffle. Il reste dans la file. Chacun a de la peinture. Ils jouent. Puis ils rincent les pinceaux ensemble. L'eau devient un peu jaune.</t>
+          <t>Nino tend la main, sans se presser. C'est à moi, le pinceau ? Oui. Victorino pose le pinceau dans le pot. Il est lourd, papa. Tu le tiens bien, Nino ? Oui, papa. La feuille est prête ? Oui, maman. Nino peint un rond jaune. C'est le soleil. Il est grand, ce rond ? Presque. Une petite tache reste près du bord. Elle est restée. Tu la laisses, Nino ? Oui, maman. Maintenant c'est toi. Une ligne ! Victorino peint une ligne, plus lente. La ligne part du rond. C'est un rayon, papa. Tu le vois, le rayon ? Oui, il part. Les pots attendent, Nino ? On fait une file. Ils posent les pots, un par un. Vite ! Victorino avance trop près. Oh. Nino refuse de foncer, cette fois. Il reste dans la file. Personne ne dit la suite à voix haute. Il regarde l'éclat de chiffon. Tu vois le point, Nino ? Oui, sur le bleu. Moi aussi. Les pots sont en file, les garçons ? Oui, maman. Chacun a de la peinture ? Oui, papa. Le ventre de Nino se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nino va vers maman. Maman, on fait quoi ? On peint, tous les deux. On attend le pinceau. Tu m'as appelée, Nino. Victorino, viens marcher jusqu'à l'évier. Victorino marche. Il pose les mains sous l'eau. L'eau est froide. Il souffle. Il se calme un peu. L'énergie est encore là. Ce n'est pas une faute. On attend. Victorino pose le pinceau dans le pot. Il attend son tour. C'est à Nino. Nino prend le grand pinceau bleu. Il peint un rond. Le rond est jaune comme un soleil. Maintenant c'est toi. Victorino peint une ligne. La ligne part du rond. C'est un rayon. Après, ils font une file pour les pots. Victorino a envie d'aller vite. On peut attendre. Victorino souffle. Il reste dans la file. Chacun a de la peinture. Ils jouent. Puis ils rincent les pinceaux ensemble. L'eau devient un peu jaune.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino tend la main, sans se presser. C'est à moi, le pinceau ? Oui. Victorino pose le pinceau dans le pot. Il est lourd, papa. Tu le tiens bien, Nino ? Oui, papa. La feuille est prête ? Oui, maman. Nino peint un rond jaune. C'est le soleil. Il est grand, ce rond ? Presque. Une petite tache reste près du bord. Elle est restée. Tu la laisses, Nino ? Oui, maman. Maintenant c'est toi. Une ligne ! Victorino peint une ligne, plus lente. La ligne part du rond. C'est un rayon, papa. Tu le vois, le rayon ? Oui, il part. Les &lt;emphasis level="moderate"&gt;pots&lt;/emphasis&gt; attendent, Nino ? On fait une file. Ils posent les pots, un par un. Vite ! Victorino avance trop près. Oh. Nino refuse de foncer, cette fois. Il reste dans la file. Personne ne dit la suite à voix haute. Il regarde l'éclat de chiffon. Tu vois le point, Nino ? Oui, sur le bleu. Moi aussi. Les pots sont en file, les garçons ? Oui, maman. Chacun a de la peinture ? Oui, papa. Le ventre de Nino se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Rayan a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Ce n'est pas une faute. Mila a pu jouer ou attendre. [pause]</t>
+          <t>Nino tend la main, sans se presser. C'est à moi, le pinceau ? Oui. Victorino pose le pinceau dans le pot. Il est lourd, papa. Tu le tiens bien, Nino ? Oui, papa. La feuille est prête ? Oui, maman. Nino peint un rond jaune. C'est le soleil. Il est grand, ce rond ? Presque. Une petite tache reste près du bord. Elle est restée. Tu la laisses, Nino ? Oui, maman. Maintenant c'est toi. Une ligne ! Victorino peint une ligne, plus lente. La ligne part du rond. C'est un rayon, papa. Tu le vois, le rayon ? Oui, il part. Les &lt;emphasis&gt;pots&lt;/emphasis&gt; attendent, Nino ? On fait une file. Ils posent les pots, un par un. Vite ! Victorino avance trop près. Oh. Nino refuse de foncer, cette fois. Il reste dans la file. Personne ne dit la suite à voix haute. Il regarde l'éclat de chiffon. Tu vois le point, Nino ? Oui, sur le bleu. Moi aussi. Les pots sont en file, les garçons ? Oui, maman. Chacun a de la peinture ? Oui, papa. Le ventre de Nino se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1631,7 +1679,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1639,10 +1687,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1665,30 +1713,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>énergie</t>
+          <t>pots</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1697,10 +1745,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1713,44 +1761,58 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_file_des_pots; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nino va vers maman.
-enfant-m|Maman, on fait quoi ?
-maman|On peint, tous les deux.
-maman|On attend le pinceau.
-maman|Tu m'as appelée, Nino.
-maman|Victorino, viens marcher jusqu'à l'évier.
-narrateur|Victorino marche.
-narrateur|Il pose les mains sous l'eau.
-narrateur|L'eau est froide.
-narrateur|Il souffle.
-narrateur|Il se calme un peu.
-papa|L'énergie est encore là.
-papa|Ce n'est pas une faute.
-enfant-m|On attend.
+          <t>narrateur|Nino tend la main, sans se presser.
+enfant-m|C'est à moi, le pinceau ?
+copain|Oui.
 narrateur|Victorino pose le pinceau dans le pot.
-narrateur|Il attend son tour.
-maman|C'est à Nino.
-narrateur|Nino prend le grand pinceau bleu.
-narrateur|Il peint un rond.
-narrateur|Le rond est jaune comme un soleil.
+enfant-m|Il est lourd, papa.
+papa|Tu le tiens bien, Nino ?
+enfant-m|Oui, papa.
+maman|La feuille est prête ?
+enfant-m|Oui, maman.
+narrateur|Nino peint un rond jaune.
+enfant-m|C'est le soleil.
+papa|Il est grand, ce rond ?
+enfant-m|Presque.
+narrateur|Une petite tache reste près du bord.
+enfant-m|Elle est restée.
+maman|Tu la laisses, Nino ?
+enfant-m|Oui, maman.
 enfant-m|Maintenant c'est toi.
-narrateur|Victorino peint une ligne.
+copain|Une ligne !
+narrateur|Victorino peint une ligne, plus lente.
 narrateur|La ligne part du rond.
-narrateur|C'est un rayon.
-narrateur|Après, ils font une file pour les pots.
-narrateur|Victorino a envie d'aller vite.
-enfant-m|On peut attendre.
-narrateur|Victorino souffle.
+enfant-m|C'est un rayon, papa.
+papa|Tu le vois, le rayon ?
+enfant-m|Oui, il part.
+maman|Les pots attendent, Nino ?
+enfant-m|On fait une file.
+narrateur|Ils posent les pots, un par un.
+copain|Vite !
+narrateur|Victorino avance trop près.
+enfant-m|Oh.
+narrateur|Nino refuse de foncer, cette fois.
 narrateur|Il reste dans la file.
-papa|Chacun a de la peinture.
-narrateur|Ils jouent.
-narrateur|Puis ils rincent les pinceaux ensemble.
-narrateur|L'eau devient un peu jaune.</t>
+narrateur|Personne ne dit la suite à voix haute.
+narrateur|Il regarde l'éclat de chiffon.
+papa|Tu vois le point, Nino ?
+enfant-m|Oui, sur le bleu.
+copain|Moi aussi.
+maman|Les pots sont en file, les garçons ?
+enfant-m|Oui, maman.
+papa|Chacun a de la peinture ?
+enfant-m|Oui, papa.
+narrateur|Le ventre de Nino se desserre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>pinceau,pots</t>
         </is>
       </c>
     </row>
@@ -1777,17 +1839,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nino et Victorino rangent les pinceaux. Vous posez les pots près du chiffon ? Oui, maman. Le rond jaune est beau. Le chiffon bleu sèche encore. On a peint ensemble. Un soleil. Nino souffle sur la feuille. La peinture brille un peu. On la laisse sécher ? Oui, papa.</t>
+          <t>Victorino glisse un pas sur le côté. Je passe ! Oh. Il veut le pinceau, sans la file. Nino ouvre la main, presque. Nino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Maman, on fait quoi ? Tu m'as appelée, Nino. Victorino, viens jusqu'à l'évier. Non. L'eau est là, tout près. Victorino marche, un peu raide. Il pose les mains sous l'eau. Elle pique ! Elle est froide, papa. L'eau de l'évier, Nino ? Oui, papa. Victorino souffle, longuement. Merci, Nino. Maman a vu les mains ouvertes. Tes pieds tiennent le sol, Victorino ? Oui. On rince les pinceaux ? Ensemble, Nino ? Oui, maman. L'eau devient un peu jaune. Elle est jaune, papa. La peinture part, Nino ? Un peu, papa. Sur le bord, un éclat de chiffon luit. L'éclat, maman ? Tu le vois, sur le bleu ? Oui, maman. Moi aussi. Le papier a failli partir. Il est resté.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nino et Victorino rangent les pinceaux. Vous posez les pots près du chiffon ? Oui, maman. Le rond jaune est beau. Le chiffon bleu sèche encore. On a peint ensemble. Un soleil. Nino souffle sur la feuille. La peinture brille un peu. On la laisse sécher ? Oui, papa.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Victorino glisse un pas sur le côté. Je passe ! Oh. Il veut le pinceau, sans la file. Nino ouvre la main, presque. Nino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Maman, on fait quoi ? Tu m'as appelée, Nino. Victorino, viens jusqu'à l'évier. Non. L'eau est là, tout près. Victorino marche, un peu raide. Il pose les mains sous l'eau. Elle pique ! Elle est froide, papa. L'eau de l'évier, Nino ? Oui, papa. Victorino souffle, longuement. Merci, Nino. Maman a vu les mains ouvertes. Tes pieds tiennent le sol, Victorino ? Oui. On rince les pinceaux ? Ensemble, Nino ? Oui, maman. L'eau devient un peu jaune. Elle est jaune, papa. La peinture part, Nino ? Un peu, papa. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat de chiffon&lt;/emphasis&gt; luit. L'éclat, maman ? Tu le vois, sur le bleu ? Oui, maman. Moi aussi. Le papier a failli partir. Il est resté.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Mila et Rayan rangent les pinceaux. Maman les attend. [pause]</t>
+          <t>&lt;low-pitch&gt;Victorino glisse un pas sur le côté. Je passe ! Oh. Il veut le pinceau, sans la file. Nino ouvre la main, presque. Nino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Maman, on fait quoi ? Tu m'as appelée, Nino. Victorino, viens jusqu'à l'évier. Non. L'eau est là, tout près. Victorino marche, un peu raide. Il pose les mains sous l'eau. Elle pique ! Elle est froide, papa. L'eau de l'évier, Nino ? Oui, papa. Victorino souffle, longuement. Merci, Nino. Maman a vu les mains ouvertes. Tes pieds tiennent le sol, Victorino ? Oui. On rince les pinceaux ? Ensemble, Nino ? Oui, maman. L'eau devient un peu jaune. Elle est jaune, papa. La peinture part, Nino ? Un peu, papa. Sur le bord, un &lt;emphasis&gt;éclat de chiffon&lt;/emphasis&gt; luit. L'éclat, maman ? Tu le vois, sur le bleu ? Oui, maman. Moi aussi. Le papier a failli partir. Il est resté.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1834,7 +1896,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1842,22 +1904,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
         <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1866,28 +1932,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de chiffon</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1896,34 +1966,69 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=victorino_veut_passer_nino_appelle_maman; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nino et Victorino rangent les pinceaux.
-maman|Vous posez les pots près du chiffon ?
+          <t>narrateur|Victorino glisse un pas sur le côté.
+copain|Je passe !
+enfant-m|Oh.
+narrateur|Il veut le pinceau, sans la file.
+narrateur|Nino ouvre la main, presque.
+narrateur|Nino refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+enfant-m|Maman, on fait quoi ?
+maman|Tu m'as appelée, Nino.
+maman|Victorino, viens jusqu'à l'évier.
+copain|Non.
+maman|L'eau est là, tout près.
+narrateur|Victorino marche, un peu raide.
+narrateur|Il pose les mains sous l'eau.
+copain|Elle pique !
+enfant-m|Elle est froide, papa.
+papa|L'eau de l'évier, Nino ?
+enfant-m|Oui, papa.
+narrateur|Victorino souffle, longuement.
+maman|Merci, Nino.
+narrateur|Maman a vu les mains ouvertes.
+papa|Tes pieds tiennent le sol, Victorino ?
+copain|Oui.
+enfant-m|On rince les pinceaux ?
+maman|Ensemble, Nino ?
 enfant-m|Oui, maman.
-papa|Le rond jaune est beau.
-narrateur|Le chiffon bleu sèche encore.
-maman|On a peint ensemble.
-enfant-m|Un soleil.
-narrateur|Nino souffle sur la feuille.
-narrateur|La peinture brille un peu.
-papa|On la laisse sécher ?
-enfant-m|Oui, papa.</t>
+narrateur|L'eau devient un peu jaune.
+enfant-m|Elle est jaune, papa.
+papa|La peinture part, Nino ?
+enfant-m|Un peu, papa.
+narrateur|Sur le bord, un éclat de chiffon luit.
+enfant-m|L'éclat, maman ?
+maman|Tu le vois, sur le bleu ?
+enfant-m|Oui, maman.
+copain|Moi aussi.
+narrateur|Le papier a failli partir.
+enfant-m|Il est resté.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>evier,eau</t>
         </is>
       </c>
     </row>
@@ -1950,17 +2055,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le soleil jaune reste sur la table. Le grand pinceau dort dans le pot bleu. Il a des rayons, maintenant. Toute la feuille.</t>
+          <t>Le soleil jaune reste sur la table. Il a des rayons, papa. Tu les vois, sur la feuille ? Oui, toute la feuille. Le grand pinceau dort dans le pot bleu. Il est calme, maman. On laisse sécher, Nino ? Oui, papa. Nino souffle sur la feuille. La peinture brille un peu. Le rond est beau. Avec la petite tache. La tache est restée, Nino ? Oui, maman. Le papier a failli partir, vous deux ? Oui, papa. Oui. Le chiffon bleu sèche près de la fenêtre. L'éclat est là, maman. Tu le vois sur le bleu ? Oui, maman. Un éclat de chiffon tient sur le bleu.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le soleil jaune reste sur la table. Le grand pinceau dort dans le pot bleu. Il a des rayons, maintenant. Toute la feuille.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le soleil jaune reste sur la table. Il a des rayons, papa. Tu les vois, sur la feuille ? Oui, toute la feuille. Le grand pinceau dort dans le pot bleu. Il est calme, maman. On laisse sécher, Nino ? Oui, papa. Nino souffle sur la feuille. La peinture brille un peu. Le rond est beau. Avec la petite tache. La tache est restée, Nino ? Oui, maman. Le papier a failli partir, vous deux ? Oui, papa. Oui. Le chiffon bleu sèche près de la fenêtre. L'éclat est là, maman. Tu le vois sur le bleu ? Oui, maman. Un &lt;emphasis level="moderate"&gt;éclat de chiffon&lt;/emphasis&gt; tient sur le bleu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le soleil jaune reste sur la table. Il a des rayons, papa. Tu les vois, sur la feuille ? Oui, toute la feuille. Le grand pinceau dort dans le pot bleu. Il est calme, maman. On laisse sécher, Nino ? Oui, papa. Nino souffle sur la feuille. La peinture brille un peu. Le rond est beau. Avec la petite tache. La tache est restée, Nino ? Oui, maman. Le papier a failli partir, vous deux ? Oui, papa. Oui. Le chiffon bleu sèche près de la fenêtre. L'éclat est là, maman. Tu le vois sur le bleu ? Oui, maman. Un &lt;emphasis&gt;éclat de chiffon&lt;/emphasis&gt; tient sur le bleu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2007,7 +2112,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2015,10 +2120,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2027,12 +2132,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2041,17 +2146,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de chiffon</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2060,11 +2169,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2073,27 +2182,54 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bleu; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
           <t>narrateur|Le soleil jaune reste sur la table.
-narrateur|Le grand pinceau dort dans le pot bleu.
-maman|Il a des rayons, maintenant.
-enfant-m|Toute la feuille.</t>
+enfant-m|Il a des rayons, papa.
+papa|Tu les vois, sur la feuille ?
+enfant-m|Oui, toute la feuille.
+maman|Le grand pinceau dort dans le pot bleu.
+enfant-m|Il est calme, maman.
+papa|On laisse sécher, Nino ?
+enfant-m|Oui, papa.
+narrateur|Nino souffle sur la feuille.
+narrateur|La peinture brille un peu.
+copain|Le rond est beau.
+enfant-m|Avec la petite tache.
+maman|La tache est restée, Nino ?
+enfant-m|Oui, maman.
+papa|Le papier a failli partir, vous deux ?
+enfant-m|Oui, papa.
+copain|Oui.
+narrateur|Le chiffon bleu sèche près de la fenêtre.
+enfant-m|L'éclat est là, maman.
+maman|Tu le vois sur le bleu ?
+enfant-m|Oui, maman.
+narrateur|Un éclat de chiffon tient sur le bleu.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>peinture,chiffon</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2171,6 +2307,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>